<commit_message>
atualizar: ajuste da planilha
</commit_message>
<xml_diff>
--- a/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
+++ b/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5011" uniqueCount="1564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5014" uniqueCount="1564">
   <si>
     <t>Data</t>
   </si>
@@ -6958,6 +6958,9 @@
       <c r="D56" s="7" t="s">
         <v>12</v>
       </c>
+      <c r="E56" s="4" t="s">
+        <v>1562</v>
+      </c>
       <c r="F56" s="4" t="s">
         <v>128</v>
       </c>
@@ -15044,6 +15047,9 @@
       <c r="D444" s="7" t="s">
         <v>733</v>
       </c>
+      <c r="E444" s="4" t="s">
+        <v>1562</v>
+      </c>
       <c r="F444" s="4" t="s">
         <v>734</v>
       </c>
@@ -15061,6 +15067,9 @@
       </c>
       <c r="D445" s="7" t="s">
         <v>727</v>
+      </c>
+      <c r="E445" s="4" t="s">
+        <v>1562</v>
       </c>
       <c r="F445" s="4" t="s">
         <v>736</v>

</xml_diff>

<commit_message>
atualizar: ajuste da planilha adicionei colunas
</commit_message>
<xml_diff>
--- a/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
+++ b/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5015" uniqueCount="1564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5024" uniqueCount="1573">
   <si>
     <t>Data</t>
   </si>
@@ -4709,6 +4709,33 @@
   </si>
   <si>
     <t>equipe</t>
+  </si>
+  <si>
+    <t>total de ocorrencia abril</t>
+  </si>
+  <si>
+    <t>total de ocorrencia maio</t>
+  </si>
+  <si>
+    <t>total de ocorrencia junho</t>
+  </si>
+  <si>
+    <t>total de ocorrencia capturada abril</t>
+  </si>
+  <si>
+    <t>total de ocorrencia capturada maio</t>
+  </si>
+  <si>
+    <t>total de ocorrencia capturada junho</t>
+  </si>
+  <si>
+    <t>% de ocorrencia capturada abril</t>
+  </si>
+  <si>
+    <t>% de ocorrencia capturada maio</t>
+  </si>
+  <si>
+    <t>% ocorrencia capturada junho</t>
   </si>
 </sst>
 </file>
@@ -4814,7 +4841,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -4874,11 +4901,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4919,9 +4956,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5229,7 +5271,16 @@
     <col min="5" max="5" width="33" style="1" customWidth="1"/>
     <col min="6" max="6" width="78.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="23" style="1" customWidth="1"/>
-    <col min="8" max="17" width="11.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.88671875" style="1" customWidth="1"/>
     <col min="18" max="25" width="9.5546875" style="1" customWidth="1"/>
     <col min="26" max="16384" width="14" style="1"/>
   </cols>
@@ -5255,6 +5306,33 @@
       <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="H3" s="28" t="s">
+        <v>1564</v>
+      </c>
+      <c r="I3" s="28" t="s">
+        <v>1565</v>
+      </c>
+      <c r="J3" s="28" t="s">
+        <v>1566</v>
+      </c>
+      <c r="K3" s="28" t="s">
+        <v>1567</v>
+      </c>
+      <c r="L3" s="28" t="s">
+        <v>1568</v>
+      </c>
+      <c r="M3" s="28" t="s">
+        <v>1569</v>
+      </c>
+      <c r="N3" s="28" t="s">
+        <v>1570</v>
+      </c>
+      <c r="O3" s="28" t="s">
+        <v>1571</v>
+      </c>
+      <c r="P3" s="28" t="s">
+        <v>1572</v>
+      </c>
     </row>
     <row r="4" spans="2:22" ht="9.75" customHeight="1">
       <c r="B4" s="3">
@@ -5273,15 +5351,36 @@
         <v>7</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
+      <c r="H4" s="5">
+        <v>2286</v>
+      </c>
+      <c r="I4" s="5">
+        <v>2019</v>
+      </c>
+      <c r="J4" s="5">
+        <v>1877</v>
+      </c>
+      <c r="K4" s="5">
+        <v>273</v>
+      </c>
+      <c r="L4" s="5">
+        <v>472</v>
+      </c>
+      <c r="M4" s="5">
+        <v>257</v>
+      </c>
+      <c r="N4" s="29">
+        <f>K4/H4</f>
+        <v>0.1194225721784777</v>
+      </c>
+      <c r="O4" s="29">
+        <f>L4/I4</f>
+        <v>0.23377909856364537</v>
+      </c>
+      <c r="P4" s="29">
+        <f>M4/J4</f>
+        <v>0.13692061800745872</v>
+      </c>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>

</xml_diff>

<commit_message>
atualizar: ajuste na planilha
</commit_message>
<xml_diff>
--- a/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
+++ b/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
@@ -13,12 +13,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">plan1!$B$3:$G$1010</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5021" uniqueCount="1570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5026" uniqueCount="1571">
   <si>
     <t>Data</t>
   </si>
@@ -4721,13 +4720,16 @@
     <t>JUNHO</t>
   </si>
   <si>
-    <t xml:space="preserve">total de ocorrencia </t>
-  </si>
-  <si>
     <t>total de ocorrencia capturadas</t>
   </si>
   <si>
     <t>% de ocorrência capturadas</t>
+  </si>
+  <si>
+    <t>total de ocorrencia registradas</t>
+  </si>
+  <si>
+    <t>total de ocorrencia recebidas</t>
   </si>
 </sst>
 </file>
@@ -4919,7 +4921,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4972,6 +4974,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5353,7 +5356,7 @@
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="28" t="s">
-        <v>1567</v>
+        <v>1569</v>
       </c>
       <c r="I4" s="5">
         <v>2286</v>
@@ -5394,7 +5397,7 @@
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="28" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
       <c r="I5" s="5">
         <v>273</v>
@@ -5437,7 +5440,7 @@
         <v>14</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="I6" s="29">
         <f>I5/I4</f>
@@ -5515,10 +5518,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
+      <c r="I8" s="30" t="s">
+        <v>1564</v>
+      </c>
+      <c r="J8" s="30" t="s">
+        <v>1565</v>
+      </c>
+      <c r="K8" s="30" t="s">
+        <v>1566</v>
+      </c>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
@@ -5550,10 +5558,21 @@
       <c r="G9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
+      <c r="H9" s="28" t="s">
+        <v>1570</v>
+      </c>
+      <c r="I9" s="34">
+        <f>100%-I10</f>
+        <v>0.88057742782152226</v>
+      </c>
+      <c r="J9" s="29">
+        <f>100%-J10</f>
+        <v>0.76622090143635457</v>
+      </c>
+      <c r="K9" s="29">
+        <f>100%-K10</f>
+        <v>0.86307938199254131</v>
+      </c>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -5586,10 +5605,18 @@
       <c r="G10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
+      <c r="H10" s="28" t="s">
+        <v>1567</v>
+      </c>
+      <c r="I10" s="29">
+        <v>0.1194225721784777</v>
+      </c>
+      <c r="J10" s="29">
+        <v>0.23377909856364537</v>
+      </c>
+      <c r="K10" s="29">
+        <v>0.13692061800745872</v>
+      </c>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>

</xml_diff>

<commit_message>
feat: adiciona suporte a Julho nos graficos, stats e sidebar + busca, paginacao e cache ETag
</commit_message>
<xml_diff>
--- a/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
+++ b/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6859" uniqueCount="2141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6861" uniqueCount="2142">
   <si>
     <t>Data</t>
   </si>
@@ -6444,6 +6444,9 @@
   </si>
   <si>
     <t>Unusual - Tixxi / CAM 83</t>
+  </si>
+  <si>
+    <t>JULHO</t>
   </si>
 </sst>
 </file>
@@ -6695,7 +6698,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6778,6 +6781,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7095,6 +7099,9 @@
       <c r="L3" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="M3" s="4" t="s">
+        <v>2141</v>
+      </c>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
@@ -7132,6 +7139,9 @@
       </c>
       <c r="L4" s="10">
         <v>1877</v>
+      </c>
+      <c r="M4" s="54">
+        <v>2530</v>
       </c>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
@@ -7175,7 +7185,9 @@
       <c r="L5" s="10">
         <v>257</v>
       </c>
-      <c r="M5" s="10"/>
+      <c r="M5" s="10">
+        <v>367</v>
+      </c>
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -7286,7 +7298,9 @@
       <c r="L8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="10"/>
+      <c r="M8" s="4" t="s">
+        <v>2141</v>
+      </c>
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
       <c r="P8" s="10"/>
@@ -7333,7 +7347,10 @@
         <f>100%-L10</f>
         <v>0.86307938199254097</v>
       </c>
-      <c r="M9" s="10"/>
+      <c r="M9" s="19">
+        <f>100%-M10</f>
+        <v>0.85494071146245054</v>
+      </c>
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
       <c r="P9" s="10"/>
@@ -7378,7 +7395,10 @@
       <c r="L10" s="19">
         <v>0.136920618007459</v>
       </c>
-      <c r="M10" s="10"/>
+      <c r="M10" s="19">
+        <f>M5/M4</f>
+        <v>0.1450592885375494</v>
+      </c>
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>

</xml_diff>